<commit_message>
Mebra: toate produsele incluse, fara ambalaje repetate
Produsele in cutie au trecut ambalajul interior (flacon 30 ml, borcan
45 ml, plic individual pansament), flaconul de 100 ml este separat pe
transparent si alb, iar seturile sunt trecute la ambalajele componentelor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VN6aeEAMfjPq2ybogLFkeD
</commit_message>
<xml_diff>
--- a/Mebra/MIRALEDO_Analiza_Ambalaje_MEBRA.xlsx
+++ b/Mebra/MIRALEDO_Analiza_Ambalaje_MEBRA.xlsx
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C21" s="130" t="inlineStr">
         <is>
-          <t>46 produse pe mebra.ro (37 individuale + 9 seturi), 28.10.2026; 15 unitati de ambalaj identificate pana acum</t>
+          <t>46 produse pe mebra.ro (37 individuale + 9 seturi), 28.10.2026; 19 unitati de ambalaj identificate</t>
         </is>
       </c>
       <c r="D21" s="131" t="n"/>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="F9" s="133" t="inlineStr">
         <is>
-          <t>MEBRA Ulei de masaj antistres 300ml; MEBRA ulei de masaj revitalizant 300ml</t>
+          <t>MEBRA Ulei de masaj antistres 300ml; MEBRA ulei de masaj revitalizant 300ml; KIT drenaj limfatic, venotonic (set)</t>
         </is>
       </c>
       <c r="G9" s="132" t="n"/>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="F11" s="133" t="inlineStr">
         <is>
-          <t>MEBRA Ulei vitaminizant copii 150ml</t>
+          <t>MEBRA Ulei vitaminizant copii 150ml; Set complet îngrijire bebeluși (set)</t>
         </is>
       </c>
       <c r="G11" s="132" t="n"/>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="F12" s="133" t="inlineStr">
         <is>
-          <t>ERITROACNOL loțiune 120ml</t>
+          <t>ERITROACNOL loțiune 120ml; KIT ten gras și acneic – extracte de plante (set)</t>
         </is>
       </c>
       <c r="G12" s="132" t="n"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C13" s="133" t="inlineStr">
         <is>
-          <t>Flacon 100 ml + spray + capac</t>
+          <t>Flacon 100 ml transparent + spray + capac</t>
         </is>
       </c>
       <c r="D13" s="133" t="inlineStr">
@@ -2462,12 +2462,12 @@
       </c>
       <c r="E13" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Transparent (flacon), alb (spray si capac), din poza</t>
         </is>
       </c>
       <c r="F13" s="133" t="inlineStr">
         <is>
-          <t>MEBRA Solutie curatare maini 100ml; MEBRA loțiune pentru picioare 100 ml; TONIFOR loțiune tonică 100ml</t>
+          <t>MEBRA Solutie curatare maini 100ml; KIT Protecție mâini + anti piele uscată (set)</t>
         </is>
       </c>
       <c r="G13" s="132" t="n"/>
@@ -2497,12 +2497,12 @@
       </c>
       <c r="C14" s="133" t="inlineStr">
         <is>
-          <t>Flacon 50 ml + spray + capac</t>
+          <t>Flacon 100 ml alb + spray + capac</t>
         </is>
       </c>
       <c r="D14" s="133" t="inlineStr">
         <is>
-          <t>50 ml</t>
+          <t>100 ml</t>
         </is>
       </c>
       <c r="E14" s="133" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="F14" s="133" t="inlineStr">
         <is>
-          <t>MEBRA spray propolis și gălbenele 50ml; MEBRA spray propolis și coada șoricelului 50ml</t>
+          <t>MEBRA loțiune pentru picioare 100 ml; TONIFOR loțiune tonică 100ml; Set complet îngrijire picioare (set); KIT anti dureri musculare (set)</t>
         </is>
       </c>
       <c r="G14" s="132" t="n"/>
@@ -2542,22 +2542,22 @@
       </c>
       <c r="C15" s="133" t="inlineStr">
         <is>
-          <t>Recipient pudra 75 g + capac</t>
+          <t>Flacon 50 ml + spray + capac</t>
         </is>
       </c>
       <c r="D15" s="133" t="inlineStr">
         <is>
-          <t>75 g</t>
+          <t>50 ml</t>
         </is>
       </c>
       <c r="E15" s="133" t="inlineStr">
         <is>
-          <t>Alb (recipient), capac colorat dupa produs, din poza</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F15" s="133" t="inlineStr">
         <is>
-          <t>MEBRA Pudră fructată 75g; MEBRA pudră mentolată 75g; MEBRA pudră propolis 75 g; MEBRA pudră mentolată împotriva transpirației 75 g; MEBRA pudră pentru copii cu portocale și cătină 75g</t>
+          <t>MEBRA spray propolis și gălbenele 50ml; MEBRA spray propolis și coada șoricelului 50ml; KIT ajutor rapid răni (set)</t>
         </is>
       </c>
       <c r="G15" s="132" t="n"/>
@@ -2587,22 +2587,22 @@
       </c>
       <c r="C16" s="133" t="inlineStr">
         <is>
-          <t>Borcan 45 ml + capac</t>
+          <t>Flacon 30 ml + spray (plastic sau sticla, in cutie)</t>
         </is>
       </c>
       <c r="D16" s="133" t="inlineStr">
         <is>
-          <t>45 ml</t>
+          <t>30 ml</t>
         </is>
       </c>
       <c r="E16" s="133" t="inlineStr">
         <is>
-          <t>Alb (borcan), capac galben / verde / rosu dupa produs, din poza</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F16" s="133" t="inlineStr">
         <is>
-          <t>MEBRA cremă cu gheara diavolului 45ml; MEBRA crema cu TATANEASA 45 ml; MEBRA cremă cu vitamina A 45ml</t>
+          <t>SALVO-MEB spray 30ml; Set sănătatea tractului respirator (set)</t>
         </is>
       </c>
       <c r="G16" s="132" t="n"/>
@@ -2632,22 +2632,22 @@
       </c>
       <c r="C17" s="133" t="inlineStr">
         <is>
-          <t>Tub 100 ml + capac</t>
+          <t>Flacon 30 ml + capac (plastic sau sticla, in cutie)</t>
         </is>
       </c>
       <c r="D17" s="133" t="inlineStr">
         <is>
-          <t>100 ml</t>
+          <t>30 ml</t>
         </is>
       </c>
       <c r="E17" s="133" t="inlineStr">
         <is>
-          <t>Alb (tub), capac rosu / galben dupa produs, din poza</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F17" s="133" t="inlineStr">
         <is>
-          <t>MEBRA cremă cu vitamina A 100ml; MEBRA cremă cu extract de gălbenele 100 ml</t>
+          <t>MEBRA TINCTURĂ PROPOLIS 30 % – supliment alimentar 30 ml; Set sănătatea tractului respirator (set)</t>
         </is>
       </c>
       <c r="G17" s="132" t="n"/>
@@ -2677,22 +2677,22 @@
       </c>
       <c r="C18" s="133" t="inlineStr">
         <is>
-          <t>Tub 75 ml + capac mare (tub asezat pe capac)</t>
+          <t>Recipient pudra 75 g + capac</t>
         </is>
       </c>
       <c r="D18" s="133" t="inlineStr">
         <is>
-          <t>75 ml</t>
+          <t>75 g</t>
         </is>
       </c>
       <c r="E18" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Alb (recipient), capac colorat dupa produs, din poza</t>
         </is>
       </c>
       <c r="F18" s="133" t="inlineStr">
         <is>
-          <t>ERITROACNOL cremă 75ml; ERITROACNOL gel 75ml</t>
+          <t>MEBRA Pudră fructată 75g; MEBRA pudră mentolată 75g; MEBRA pudră propolis 75 g; MEBRA pudră mentolată împotriva transpirației 75 g; MEBRA pudră pentru copii cu portocale și cătină 75g; Set complet îngrijire bebeluși (set)</t>
         </is>
       </c>
       <c r="G18" s="132" t="n"/>
@@ -2722,22 +2722,22 @@
       </c>
       <c r="C19" s="133" t="inlineStr">
         <is>
-          <t>Tub 75 ml + capac</t>
+          <t>Borcan 45 ml + capac</t>
         </is>
       </c>
       <c r="D19" s="133" t="inlineStr">
         <is>
-          <t>75 ml</t>
+          <t>45 ml</t>
         </is>
       </c>
       <c r="E19" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Alb (borcan), capac galben / verde / rosu dupa produs, din poza</t>
         </is>
       </c>
       <c r="F19" s="133" t="inlineStr">
         <is>
-          <t>MEBRA balsam pentru picioare obosite 75ml; TONIFOR cremă tonică și relaxantă 75ml; MEBRA crema cu extract de CASTANE 75ml; TONIFOR arnica gel 75ml</t>
+          <t>MEBRA cremă cu gheara diavolului 45ml; MEBRA crema cu TATANEASA 45 ml; MEBRA cremă cu vitamina A 45ml; MEDARA cremă cu vitaminele A și E 45 ml (pe site doar cutia, borcanul de confirmat); KIT îngrijire iarnă, piele ultra uscată (set)</t>
         </is>
       </c>
       <c r="G19" s="132" t="n"/>
@@ -2767,22 +2767,22 @@
       </c>
       <c r="C20" s="133" t="inlineStr">
         <is>
-          <t>Tub 40 ml + capac</t>
+          <t>Tub 100 ml + capac</t>
         </is>
       </c>
       <c r="D20" s="133" t="inlineStr">
         <is>
-          <t>40 ml</t>
+          <t>100 ml</t>
         </is>
       </c>
       <c r="E20" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Alb (tub), capac rosu / galben dupa produs, din poza</t>
         </is>
       </c>
       <c r="F20" s="133" t="inlineStr">
         <is>
-          <t>MEBRA cremă cu vitamina A 40ml; MEBRA Cremă îngrijire călcâie 40ml</t>
+          <t>MEBRA cremă cu vitamina A 100ml; MEBRA cremă cu extract de gălbenele 100 ml</t>
         </is>
       </c>
       <c r="G20" s="132" t="n"/>
@@ -2812,12 +2812,12 @@
       </c>
       <c r="C21" s="133" t="inlineStr">
         <is>
-          <t>Recipient aerosol 59,5 g + valva + capac (in cutie)</t>
+          <t>Tub 75 ml + capac mare (tub asezat pe capac)</t>
         </is>
       </c>
       <c r="D21" s="133" t="inlineStr">
         <is>
-          <t>59,5 g</t>
+          <t>75 ml</t>
         </is>
       </c>
       <c r="E21" s="133" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="F21" s="133" t="inlineStr">
         <is>
-          <t>OXIMED Spray cutanat 59,5g</t>
+          <t>ERITROACNOL cremă 75ml; ERITROACNOL gel 75ml; KIT ten gras și acneic – extracte de plante (set)</t>
         </is>
       </c>
       <c r="G21" s="132" t="n"/>
@@ -2851,79 +2851,255 @@
       </c>
       <c r="M21" s="138" t="n"/>
     </row>
-    <row r="22" s="128"/>
-    <row r="23" s="128"/>
-    <row r="24" ht="19.95" customHeight="1" s="128">
-      <c r="C24" s="76" t="inlineStr">
+    <row r="22" s="128">
+      <c r="B22" s="132" t="n">
+        <v>16</v>
+      </c>
+      <c r="C22" s="133" t="inlineStr">
+        <is>
+          <t>Tub 75 ml + capac</t>
+        </is>
+      </c>
+      <c r="D22" s="133" t="inlineStr">
+        <is>
+          <t>75 ml</t>
+        </is>
+      </c>
+      <c r="E22" s="133" t="inlineStr">
+        <is>
+          <t>Alb (din poza)</t>
+        </is>
+      </c>
+      <c r="F22" s="133" t="inlineStr">
+        <is>
+          <t>MEBRA balsam pentru picioare obosite 75ml; TONIFOR cremă tonică și relaxantă 75ml; MEBRA crema cu extract de CASTANE 75ml; TONIFOR arnica gel 75ml; Set complet îngrijire picioare (set); KIT drenaj limfatic, venotonic (set); KIT anti dureri musculare (set)</t>
+        </is>
+      </c>
+      <c r="G22" s="132" t="n"/>
+      <c r="H22" s="134">
+        <f>IFERROR(INDIRECT("'"&amp;G22&amp;"'!E26"),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="135">
+        <f>IFERROR(INDIRECT("'"&amp;G22&amp;"'!E27"),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="136">
+        <f>IFERROR(INDIRECT("'"&amp;G22&amp;"'!E28"),"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="137" t="n"/>
+      <c r="L22" s="137" t="inlineStr">
+        <is>
+          <t>In curs</t>
+        </is>
+      </c>
+      <c r="M22" s="138" t="n"/>
+    </row>
+    <row r="23" s="128">
+      <c r="B23" s="132" t="n">
+        <v>17</v>
+      </c>
+      <c r="C23" s="133" t="inlineStr">
+        <is>
+          <t>Tub 40 ml + capac</t>
+        </is>
+      </c>
+      <c r="D23" s="133" t="inlineStr">
+        <is>
+          <t>40 ml</t>
+        </is>
+      </c>
+      <c r="E23" s="133" t="inlineStr">
+        <is>
+          <t>Alb (din poza)</t>
+        </is>
+      </c>
+      <c r="F23" s="133" t="inlineStr">
+        <is>
+          <t>MEBRA cremă cu vitamina A 40ml; MEBRA Cremă îngrijire călcâie 40ml; KIT Protecție mâini + anti piele uscată (set); KIT îngrijire iarnă, piele ultra uscată (set)</t>
+        </is>
+      </c>
+      <c r="G23" s="132" t="n"/>
+      <c r="H23" s="134">
+        <f>IFERROR(INDIRECT("'"&amp;G23&amp;"'!E26"),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="135">
+        <f>IFERROR(INDIRECT("'"&amp;G23&amp;"'!E27"),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="136">
+        <f>IFERROR(INDIRECT("'"&amp;G23&amp;"'!E28"),"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="137" t="n"/>
+      <c r="L23" s="137" t="inlineStr">
+        <is>
+          <t>In curs</t>
+        </is>
+      </c>
+      <c r="M23" s="138" t="n"/>
+    </row>
+    <row r="24" s="128">
+      <c r="B24" s="132" t="n">
+        <v>18</v>
+      </c>
+      <c r="C24" s="133" t="inlineStr">
+        <is>
+          <t>Plic individual pansament 19x72 mm (in cutie)</t>
+        </is>
+      </c>
+      <c r="D24" s="133" t="inlineStr">
+        <is>
+          <t>De confirmat</t>
+        </is>
+      </c>
+      <c r="E24" s="133" t="inlineStr">
+        <is>
+          <t>Alb cu imprimare rosie (din poza)</t>
+        </is>
+      </c>
+      <c r="F24" s="133" t="inlineStr">
+        <is>
+          <t>Pansament rezistent la apa 207M, 1.9 cm*7.2 cm set 20 bucati; KIT ajutor rapid răni (set)</t>
+        </is>
+      </c>
+      <c r="G24" s="132" t="n"/>
+      <c r="H24" s="134">
+        <f>IFERROR(INDIRECT("'"&amp;G24&amp;"'!E26"),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="135">
+        <f>IFERROR(INDIRECT("'"&amp;G24&amp;"'!E27"),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="136">
+        <f>IFERROR(INDIRECT("'"&amp;G24&amp;"'!E28"),"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="137" t="n"/>
+      <c r="L24" s="137" t="inlineStr">
+        <is>
+          <t>In curs</t>
+        </is>
+      </c>
+      <c r="M24" s="138" t="n"/>
+    </row>
+    <row r="25" s="128">
+      <c r="B25" s="132" t="n">
+        <v>19</v>
+      </c>
+      <c r="C25" s="133" t="inlineStr">
+        <is>
+          <t>Recipient aerosol 59,5 g + valva + capac (in cutie)</t>
+        </is>
+      </c>
+      <c r="D25" s="133" t="inlineStr">
+        <is>
+          <t>59,5 g</t>
+        </is>
+      </c>
+      <c r="E25" s="133" t="inlineStr">
+        <is>
+          <t>Alb (din poza)</t>
+        </is>
+      </c>
+      <c r="F25" s="133" t="inlineStr">
+        <is>
+          <t>OXIMED Spray cutanat 59,5g</t>
+        </is>
+      </c>
+      <c r="G25" s="132" t="n"/>
+      <c r="H25" s="134">
+        <f>IFERROR(INDIRECT("'"&amp;G25&amp;"'!E26"),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="135">
+        <f>IFERROR(INDIRECT("'"&amp;G25&amp;"'!E27"),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="136">
+        <f>IFERROR(INDIRECT("'"&amp;G25&amp;"'!E28"),"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="137" t="n"/>
+      <c r="L25" s="137" t="inlineStr">
+        <is>
+          <t>In curs</t>
+        </is>
+      </c>
+      <c r="M25" s="138" t="n"/>
+    </row>
+    <row r="26" s="128"/>
+    <row r="27" s="128"/>
+    <row r="28" ht="19.95" customHeight="1" s="128">
+      <c r="C28" s="76" t="inlineStr">
         <is>
           <t>Rezumat (automat)</t>
         </is>
       </c>
-      <c r="D24" s="73" t="inlineStr">
+      <c r="D28" s="73" t="inlineStr">
         <is>
           <t>Nr. unitati</t>
         </is>
-      </c>
-    </row>
-    <row r="25" ht="19.95" customHeight="1" s="128">
-      <c r="C25" s="74" t="inlineStr">
-        <is>
-          <t>Unitati analizate</t>
-        </is>
-      </c>
-      <c r="D25" s="75">
-        <f>COUNTIF(G7:G21,"?*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="19.95" customHeight="1" s="128">
-      <c r="C26" s="74" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D26" s="75">
-        <f>COUNTIF($J$7:$J$21,C26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="19.95" customHeight="1" s="128">
-      <c r="C27" s="74" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D27" s="75">
-        <f>COUNTIF($J$7:$J$21,C27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="19.95" customHeight="1" s="128">
-      <c r="C28" s="74" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D28" s="75">
-        <f>COUNTIF($J$7:$J$21,C28)</f>
-        <v/>
       </c>
     </row>
     <row r="29" ht="19.95" customHeight="1" s="128">
       <c r="C29" s="74" t="inlineStr">
         <is>
+          <t>Unitati analizate</t>
+        </is>
+      </c>
+      <c r="D29" s="75">
+        <f>COUNTIF(G7:G25,"?*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="19.95" customHeight="1" s="128">
+      <c r="C30" s="74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D30" s="75">
+        <f>COUNTIF($J$7:$J$25,C30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="19.95" customHeight="1" s="128">
+      <c r="C31" s="74" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D31" s="75">
+        <f>COUNTIF($J$7:$J$25,C31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="19.95" customHeight="1" s="128">
+      <c r="C32" s="74" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D32" s="75">
+        <f>COUNTIF($J$7:$J$25,C32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="19.95" customHeight="1" s="128">
+      <c r="C33" s="74" t="inlineStr">
+        <is>
           <t>Sub 70% - nereciclabil</t>
         </is>
       </c>
-      <c r="D29" s="75">
-        <f>COUNTIF($J$7:$J$21,C29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
+      <c r="D33" s="75">
+        <f>COUNTIF($J$7:$J$25,C33)</f>
+        <v/>
+      </c>
+    </row>
     <row r="34"/>
     <row r="35"/>
     <row r="36"/>
@@ -2935,12 +3111,12 @@
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="B2:K2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G7:G21">
+  <conditionalFormatting sqref="G7:G25">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND($G7&lt;&gt;"",$H7="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J21">
+  <conditionalFormatting sqref="J7:J25">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>OR($J7="A",$J7="B")</formula>
     </cfRule>
@@ -2952,10 +3128,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K7:K21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Prioritate" error="Alegeti: Mare, Medie sau Mica." type="list">
+    <dataValidation sqref="K7:K25" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Prioritate" error="Alegeti: Mare, Medie sau Mica." type="list">
       <formula1>"Mare,Medie,Mica"</formula1>
     </dataValidation>
-    <dataValidation sqref="L7:L21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Stadiu analiza" error="Valoarea nu este in lista. Puteti continua daca este intentionat." type="list" errorStyle="information">
+    <dataValidation sqref="L7:L25" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Stadiu analiza" error="Valoarea nu este in lista. Puteti continua daca este intentionat." type="list" errorStyle="information">
       <formula1>"Identificata,In completare,Completa,Oferta trimisa"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>